<commit_message>
Fix V2.1 payer acceptance workbook percentages
</commit_message>
<xml_diff>
--- a/data/synthetic/v2_1/payer_mix_acceptance.xlsx
+++ b/data/synthetic/v2_1/payer_mix_acceptance.xlsx
@@ -60,9 +60,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,66 +429,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Entity ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Clinic</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>FTE Count</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Work Days</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Visits Per Day</t>
-        </is>
-      </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Visits Per Provider Day</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Utilization</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Rev / Visit</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Variable Labor Cost Per Visit</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Variable Supply Cost Per Visit</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Fixed Operating Expense</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Reimbursement Factor</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Currency</t>
         </is>
@@ -496,42 +502,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>NSC</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Nashville Specialty Clinic</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>4</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>22</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>18</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>195</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>55</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>18</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>85000</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>1</v>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
@@ -540,42 +551,47 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>NSC</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Nashville Specialty Clinic</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>4</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>22</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>18</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>195</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>55</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>18</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>85000</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>1</v>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
@@ -639,17 +655,17 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>42</v>
-      </c>
-      <c r="D2" t="n">
-        <v>31</v>
-      </c>
-      <c r="E2" t="n">
-        <v>12</v>
-      </c>
-      <c r="F2" t="n">
-        <v>15</v>
+      <c r="C2" s="2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="3">
@@ -663,17 +679,17 @@
           <t>2026-09</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>40</v>
-      </c>
-      <c r="D3" t="n">
-        <v>33</v>
-      </c>
-      <c r="E3" t="n">
-        <v>12</v>
-      </c>
-      <c r="F3" t="n">
-        <v>15</v>
+      <c r="C3" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0.15</v>
       </c>
     </row>
   </sheetData>
@@ -759,17 +775,17 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>42</v>
-      </c>
-      <c r="D2" t="n">
-        <v>31</v>
-      </c>
-      <c r="E2" t="n">
-        <v>12</v>
-      </c>
-      <c r="F2" t="n">
-        <v>15</v>
+      <c r="C2" s="2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0.15</v>
       </c>
       <c r="G2" t="n">
         <v>240</v>
@@ -800,17 +816,17 @@
           <t>2026-09</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>40</v>
-      </c>
-      <c r="D3" t="n">
-        <v>33</v>
-      </c>
-      <c r="E3" t="n">
-        <v>12</v>
-      </c>
-      <c r="F3" t="n">
-        <v>15</v>
+      <c r="C3" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0.15</v>
       </c>
       <c r="G3" t="n">
         <v>245</v>

</xml_diff>